<commit_message>
Add Phase4 projects: Mean Finder and Zero-Crossing custom AXI IP with documentation
</commit_message>
<xml_diff>
--- a/fpga-soc-learning/FIR_Design_Reference_Table.xlsx
+++ b/fpga-soc-learning/FIR_Design_Reference_Table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Embedded-System-Portfolio-Projects\fpga-soc-learning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7F88687-9AEA-4310-A12E-F7201F117DFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F54E23E-E670-477C-8197-955BC32ED34F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-104" yWindow="-104" windowWidth="22326" windowHeight="11947" tabRatio="500" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -299,9 +299,6 @@
     <t>&gt;= 33 bits (our case), use 40 bits</t>
   </si>
   <si>
-    <t>40 bits ✅</t>
-  </si>
-  <si>
     <t>14</t>
   </si>
   <si>
@@ -371,9 +368,6 @@
     <t>N DSP48 used (not in LUT section)</t>
   </si>
   <si>
-    <t>8 DSP48</t>
-  </si>
-  <si>
     <t>18</t>
   </si>
   <si>
@@ -387,9 +381,6 @@
   </si>
   <si>
     <t>N/2 DSP48 blocks (vs N without)</t>
-  </si>
-  <si>
-    <t>4 DSP48 optimized</t>
   </si>
   <si>
     <t>19</t>
@@ -1053,13 +1044,22 @@
   </si>
   <si>
     <t>7958 &lt; 32767 ✅</t>
+  </si>
+  <si>
+    <t>42 bits ✅</t>
+  </si>
+  <si>
+    <t>32 DSP48</t>
+  </si>
+  <si>
+    <t>16 DSP48 optimized</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1202,6 +1202,13 @@
       <color rgb="FF2E75B6"/>
       <name val="Arial"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1E4620"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="16">
@@ -1437,7 +1444,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1656,6 +1663,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2012,10 +2022,10 @@
         <v>14</v>
       </c>
       <c r="G6" s="25" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="H6" s="26" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="I6" s="19"/>
     </row>
@@ -2037,7 +2047,7 @@
         <v>20</v>
       </c>
       <c r="G7" s="25" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="H7" s="26"/>
       <c r="I7" s="27"/>
@@ -2060,7 +2070,7 @@
         <v>26</v>
       </c>
       <c r="G8" s="25" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="H8" s="26"/>
       <c r="I8" s="19"/>
@@ -2083,7 +2093,7 @@
         <v>32</v>
       </c>
       <c r="G9" s="25" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="H9" s="26"/>
       <c r="I9" s="27"/>
@@ -2106,7 +2116,7 @@
         <v>38</v>
       </c>
       <c r="G10" s="25" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="H10" s="26"/>
       <c r="I10" s="19"/>
@@ -2129,7 +2139,7 @@
         <v>44</v>
       </c>
       <c r="G11" s="25" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="H11" s="26"/>
       <c r="I11" s="27"/>
@@ -2152,7 +2162,7 @@
         <v>50</v>
       </c>
       <c r="G12" s="25" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="H12" s="26"/>
       <c r="I12" s="19"/>
@@ -2188,7 +2198,7 @@
         <v>56</v>
       </c>
       <c r="G15" s="25" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="H15" s="26" t="b">
         <v>1</v>
@@ -2216,7 +2226,7 @@
         <v>62</v>
       </c>
       <c r="H16" s="26" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="I16" s="19"/>
     </row>
@@ -2238,7 +2248,7 @@
         <v>67</v>
       </c>
       <c r="G17" s="25" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="H17" s="26" t="b">
         <v>1</v>
@@ -2325,8 +2335,8 @@
       <c r="F22" s="24" t="s">
         <v>85</v>
       </c>
-      <c r="G22" s="25" t="s">
-        <v>86</v>
+      <c r="G22" s="81" t="s">
+        <v>334</v>
       </c>
       <c r="H22" s="26"/>
       <c r="I22" s="19"/>
@@ -2334,47 +2344,47 @@
     <row r="23" spans="1:9" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="27"/>
       <c r="B23" s="28" t="s">
+        <v>86</v>
+      </c>
+      <c r="C23" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="C23" s="29" t="s">
+      <c r="D23" s="30" t="s">
         <v>88</v>
       </c>
-      <c r="D23" s="30" t="s">
+      <c r="E23" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="E23" s="31" t="s">
+      <c r="F23" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="F23" s="24" t="s">
+      <c r="G23" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="G23" s="25" t="s">
-        <v>92</v>
-      </c>
       <c r="H23" s="26" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="I23" s="27"/>
     </row>
     <row r="24" spans="1:9" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="19"/>
       <c r="B24" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="C24" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="C24" s="21" t="s">
+      <c r="D24" s="22" t="s">
         <v>94</v>
       </c>
-      <c r="D24" s="22" t="s">
+      <c r="E24" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="E24" s="23" t="s">
+      <c r="F24" s="24" t="s">
         <v>96</v>
       </c>
-      <c r="F24" s="24" t="s">
+      <c r="G24" s="25" t="s">
         <v>97</v>
-      </c>
-      <c r="G24" s="25" t="s">
-        <v>98</v>
       </c>
       <c r="H24" s="26"/>
       <c r="I24" s="19"/>
@@ -2382,22 +2392,22 @@
     <row r="25" spans="1:9" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="27"/>
       <c r="B25" s="28" t="s">
+        <v>98</v>
+      </c>
+      <c r="C25" s="29" t="s">
         <v>99</v>
       </c>
-      <c r="C25" s="29" t="s">
+      <c r="D25" s="30" t="s">
         <v>100</v>
       </c>
-      <c r="D25" s="30" t="s">
+      <c r="E25" s="31" t="s">
         <v>101</v>
       </c>
-      <c r="E25" s="31" t="s">
+      <c r="F25" s="24" t="s">
         <v>102</v>
       </c>
-      <c r="F25" s="24" t="s">
+      <c r="G25" s="25" t="s">
         <v>103</v>
-      </c>
-      <c r="G25" s="25" t="s">
-        <v>104</v>
       </c>
       <c r="H25" s="26"/>
       <c r="I25" s="27"/>
@@ -2405,22 +2415,22 @@
     <row r="26" spans="1:9" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="19"/>
       <c r="B26" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="C26" s="21" t="s">
         <v>105</v>
       </c>
-      <c r="C26" s="21" t="s">
+      <c r="D26" s="22" t="s">
         <v>106</v>
       </c>
-      <c r="D26" s="22" t="s">
+      <c r="E26" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="E26" s="23" t="s">
+      <c r="F26" s="24" t="s">
         <v>108</v>
       </c>
-      <c r="F26" s="24" t="s">
-        <v>109</v>
-      </c>
-      <c r="G26" s="25" t="s">
-        <v>110</v>
+      <c r="G26" s="81" t="s">
+        <v>335</v>
       </c>
       <c r="H26" s="26"/>
       <c r="I26" s="19"/>
@@ -2428,22 +2438,22 @@
     <row r="27" spans="1:9" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="27"/>
       <c r="B27" s="28" t="s">
+        <v>109</v>
+      </c>
+      <c r="C27" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="D27" s="30" t="s">
         <v>111</v>
       </c>
-      <c r="C27" s="29" t="s">
+      <c r="E27" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="D27" s="30" t="s">
+      <c r="F27" s="24" t="s">
         <v>113</v>
       </c>
-      <c r="E27" s="31" t="s">
-        <v>114</v>
-      </c>
-      <c r="F27" s="24" t="s">
-        <v>115</v>
-      </c>
-      <c r="G27" s="25" t="s">
-        <v>116</v>
+      <c r="G27" s="81" t="s">
+        <v>336</v>
       </c>
       <c r="H27" s="26"/>
       <c r="I27" s="27"/>
@@ -2451,22 +2461,22 @@
     <row r="28" spans="1:9" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="19"/>
       <c r="B28" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="C28" s="21" t="s">
+        <v>115</v>
+      </c>
+      <c r="D28" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="E28" s="23" t="s">
         <v>117</v>
       </c>
-      <c r="C28" s="21" t="s">
+      <c r="F28" s="24" t="s">
         <v>118</v>
       </c>
-      <c r="D28" s="22" t="s">
+      <c r="G28" s="25" t="s">
         <v>119</v>
-      </c>
-      <c r="E28" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="F28" s="24" t="s">
-        <v>121</v>
-      </c>
-      <c r="G28" s="25" t="s">
-        <v>122</v>
       </c>
       <c r="H28" s="26"/>
       <c r="I28" s="19"/>
@@ -2474,22 +2484,22 @@
     <row r="29" spans="1:9" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="27"/>
       <c r="B29" s="28" t="s">
+        <v>120</v>
+      </c>
+      <c r="C29" s="29" t="s">
+        <v>121</v>
+      </c>
+      <c r="D29" s="30" t="s">
+        <v>122</v>
+      </c>
+      <c r="E29" s="31" t="s">
         <v>123</v>
       </c>
-      <c r="C29" s="29" t="s">
+      <c r="F29" s="24" t="s">
         <v>124</v>
       </c>
-      <c r="D29" s="30" t="s">
+      <c r="G29" s="25" t="s">
         <v>125</v>
-      </c>
-      <c r="E29" s="31" t="s">
-        <v>126</v>
-      </c>
-      <c r="F29" s="24" t="s">
-        <v>127</v>
-      </c>
-      <c r="G29" s="25" t="s">
-        <v>128</v>
       </c>
       <c r="H29" s="26"/>
       <c r="I29" s="27"/>
@@ -2497,7 +2507,7 @@
     <row r="31" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="34"/>
       <c r="B31" s="9" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C31" s="9"/>
       <c r="D31" s="9"/>
@@ -2510,22 +2520,22 @@
     <row r="32" spans="1:9" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="19"/>
       <c r="B32" s="20" t="s">
+        <v>127</v>
+      </c>
+      <c r="C32" s="21" t="s">
+        <v>128</v>
+      </c>
+      <c r="D32" s="22" t="s">
+        <v>129</v>
+      </c>
+      <c r="E32" s="23" t="s">
         <v>130</v>
       </c>
-      <c r="C32" s="21" t="s">
+      <c r="F32" s="24" t="s">
         <v>131</v>
       </c>
-      <c r="D32" s="22" t="s">
+      <c r="G32" s="25" t="s">
         <v>132</v>
-      </c>
-      <c r="E32" s="23" t="s">
-        <v>133</v>
-      </c>
-      <c r="F32" s="24" t="s">
-        <v>134</v>
-      </c>
-      <c r="G32" s="25" t="s">
-        <v>135</v>
       </c>
       <c r="H32" s="26"/>
       <c r="I32" s="19"/>
@@ -2533,22 +2543,22 @@
     <row r="33" spans="1:9" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="27"/>
       <c r="B33" s="28" t="s">
+        <v>133</v>
+      </c>
+      <c r="C33" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="D33" s="30" t="s">
+        <v>135</v>
+      </c>
+      <c r="E33" s="31" t="s">
         <v>136</v>
       </c>
-      <c r="C33" s="29" t="s">
+      <c r="F33" s="24" t="s">
         <v>137</v>
       </c>
-      <c r="D33" s="30" t="s">
+      <c r="G33" s="25" t="s">
         <v>138</v>
-      </c>
-      <c r="E33" s="31" t="s">
-        <v>139</v>
-      </c>
-      <c r="F33" s="24" t="s">
-        <v>140</v>
-      </c>
-      <c r="G33" s="25" t="s">
-        <v>141</v>
       </c>
       <c r="H33" s="26"/>
       <c r="I33" s="27"/>
@@ -2556,22 +2566,22 @@
     <row r="34" spans="1:9" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="19"/>
       <c r="B34" s="20" t="s">
+        <v>139</v>
+      </c>
+      <c r="C34" s="21" t="s">
+        <v>140</v>
+      </c>
+      <c r="D34" s="22" t="s">
+        <v>141</v>
+      </c>
+      <c r="E34" s="23" t="s">
         <v>142</v>
       </c>
-      <c r="C34" s="21" t="s">
+      <c r="F34" s="24" t="s">
         <v>143</v>
       </c>
-      <c r="D34" s="22" t="s">
+      <c r="G34" s="25" t="s">
         <v>144</v>
-      </c>
-      <c r="E34" s="23" t="s">
-        <v>145</v>
-      </c>
-      <c r="F34" s="24" t="s">
-        <v>146</v>
-      </c>
-      <c r="G34" s="25" t="s">
-        <v>147</v>
       </c>
       <c r="H34" s="26"/>
       <c r="I34" s="19"/>
@@ -2579,22 +2589,22 @@
     <row r="35" spans="1:9" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="27"/>
       <c r="B35" s="28" t="s">
+        <v>145</v>
+      </c>
+      <c r="C35" s="29" t="s">
+        <v>146</v>
+      </c>
+      <c r="D35" s="30" t="s">
+        <v>147</v>
+      </c>
+      <c r="E35" s="31" t="s">
         <v>148</v>
       </c>
-      <c r="C35" s="29" t="s">
+      <c r="F35" s="24" t="s">
         <v>149</v>
       </c>
-      <c r="D35" s="30" t="s">
-        <v>150</v>
-      </c>
-      <c r="E35" s="31" t="s">
-        <v>151</v>
-      </c>
-      <c r="F35" s="24" t="s">
-        <v>152</v>
-      </c>
       <c r="G35" s="25" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H35" s="26"/>
       <c r="I35" s="27"/>
@@ -2602,29 +2612,29 @@
     <row r="36" spans="1:9" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="19"/>
       <c r="B36" s="20" t="s">
+        <v>150</v>
+      </c>
+      <c r="C36" s="21" t="s">
+        <v>151</v>
+      </c>
+      <c r="D36" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="E36" s="23" t="s">
         <v>153</v>
       </c>
-      <c r="C36" s="21" t="s">
+      <c r="F36" s="24" t="s">
         <v>154</v>
       </c>
-      <c r="D36" s="22" t="s">
+      <c r="G36" s="25" t="s">
         <v>155</v>
-      </c>
-      <c r="E36" s="23" t="s">
-        <v>156</v>
-      </c>
-      <c r="F36" s="24" t="s">
-        <v>157</v>
-      </c>
-      <c r="G36" s="25" t="s">
-        <v>158</v>
       </c>
       <c r="H36" s="26"/>
       <c r="I36" s="19"/>
     </row>
     <row r="38" spans="1:9" ht="19.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="8" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C38" s="8"/>
       <c r="D38" s="8"/>
@@ -2662,7 +2672,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="14" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="C1" s="14"/>
       <c r="D1" s="14"/>
@@ -2670,7 +2680,7 @@
     </row>
     <row r="2" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="13" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>
@@ -2683,19 +2693,19 @@
         <v>2</v>
       </c>
       <c r="C4" s="35" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D4" s="35" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="E4" s="35" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="18"/>
       <c r="B5" s="7" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
@@ -2714,7 +2724,7 @@
         <v>15</v>
       </c>
       <c r="E7" s="36" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="F7" s="19"/>
     </row>
@@ -2724,13 +2734,13 @@
         <v>16</v>
       </c>
       <c r="C8" s="29" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="D8" s="25" t="s">
         <v>21</v>
       </c>
       <c r="E8" s="37" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F8" s="27"/>
     </row>
@@ -2740,13 +2750,13 @@
         <v>22</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="D9" s="25" t="s">
         <v>27</v>
       </c>
       <c r="E9" s="36" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="F9" s="19"/>
     </row>
@@ -2756,13 +2766,13 @@
         <v>28</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="D10" s="25" t="s">
         <v>33</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="F10" s="27"/>
     </row>
@@ -2778,7 +2788,7 @@
         <v>39</v>
       </c>
       <c r="E11" s="36" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F11" s="19"/>
     </row>
@@ -2794,7 +2804,7 @@
         <v>45</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="F12" s="27"/>
     </row>
@@ -2807,17 +2817,17 @@
         <v>47</v>
       </c>
       <c r="D13" s="25" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="E13" s="36" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="F13" s="19"/>
     </row>
     <row r="15" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="32"/>
       <c r="B15" s="6" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="C15" s="6"/>
       <c r="D15" s="6"/>
@@ -2830,13 +2840,13 @@
         <v>52</v>
       </c>
       <c r="C17" s="29" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="D17" s="25" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="E17" s="37" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="F17" s="27"/>
     </row>
@@ -2846,13 +2856,13 @@
         <v>57</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="D18" s="25" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="E18" s="36" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F18" s="19"/>
     </row>
@@ -2862,13 +2872,13 @@
         <v>63</v>
       </c>
       <c r="C19" s="29" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="D19" s="25" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="E19" s="37" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="F19" s="27"/>
     </row>
@@ -2878,13 +2888,13 @@
         <v>68</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="D20" s="25" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="E20" s="36" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="F20" s="19"/>
     </row>
@@ -2894,13 +2904,13 @@
         <v>74</v>
       </c>
       <c r="C21" s="29" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="D21" s="25" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="E21" s="37" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="F21" s="27"/>
     </row>
@@ -2913,33 +2923,33 @@
         <v>64</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="E22" s="36" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="F22" s="19"/>
     </row>
     <row r="23" spans="1:6" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="27"/>
       <c r="B23" s="28" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C23" s="29" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="E23" s="37" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="F23" s="27"/>
     </row>
     <row r="25" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="33"/>
       <c r="B25" s="5" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C25" s="5"/>
       <c r="D25" s="5"/>
@@ -2949,160 +2959,160 @@
     <row r="27" spans="1:6" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="19"/>
       <c r="B27" s="20" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D27" s="25" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="E27" s="36" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="F27" s="19"/>
     </row>
     <row r="28" spans="1:6" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="27"/>
       <c r="B28" s="28" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C28" s="29" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D28" s="25" t="s">
+        <v>197</v>
+      </c>
+      <c r="E28" s="37" t="s">
         <v>200</v>
-      </c>
-      <c r="E28" s="37" t="s">
-        <v>203</v>
       </c>
       <c r="F28" s="27"/>
     </row>
     <row r="29" spans="1:6" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="19"/>
       <c r="B29" s="20" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="D29" s="25" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E29" s="36" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="F29" s="19"/>
     </row>
     <row r="30" spans="1:6" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="27"/>
       <c r="B30" s="28" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C30" s="29" t="s">
         <v>82</v>
       </c>
       <c r="D30" s="25" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="E30" s="37" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="F30" s="27"/>
     </row>
     <row r="31" spans="1:6" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="19"/>
       <c r="B31" s="20" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="D31" s="25" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="E31" s="36" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="F31" s="19"/>
     </row>
     <row r="32" spans="1:6" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="27"/>
       <c r="B32" s="28" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C32" s="29" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D32" s="25" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="E32" s="37" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="F32" s="27"/>
     </row>
     <row r="33" spans="1:6" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="19"/>
       <c r="B33" s="20" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C33" s="21" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="D33" s="25" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E33" s="36" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="F33" s="19"/>
     </row>
     <row r="34" spans="1:6" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="27"/>
       <c r="B34" s="28" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C34" s="29" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="D34" s="25" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="E34" s="37" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="F34" s="27"/>
     </row>
     <row r="35" spans="1:6" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="19"/>
       <c r="B35" s="20" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C35" s="21" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="D35" s="25" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="E35" s="36" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="F35" s="19"/>
     </row>
     <row r="36" spans="1:6" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="27"/>
       <c r="B36" s="28" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C36" s="29" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="D36" s="25" t="s">
         <v>15</v>
       </c>
       <c r="E36" s="37" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="F36" s="27"/>
     </row>
@@ -3135,7 +3145,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="14" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="C1" s="14"/>
       <c r="D1" s="14"/>
@@ -3145,7 +3155,7 @@
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="13" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>
@@ -3157,247 +3167,247 @@
     <row r="4" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="35"/>
       <c r="B4" s="35" t="s">
+        <v>225</v>
+      </c>
+      <c r="C4" s="35" t="s">
+        <v>226</v>
+      </c>
+      <c r="D4" s="35" t="s">
+        <v>227</v>
+      </c>
+      <c r="E4" s="35" t="s">
         <v>228</v>
       </c>
-      <c r="C4" s="35" t="s">
+      <c r="F4" s="35" t="s">
         <v>229</v>
       </c>
-      <c r="D4" s="35" t="s">
+      <c r="G4" s="35" t="s">
         <v>230</v>
-      </c>
-      <c r="E4" s="35" t="s">
-        <v>231</v>
-      </c>
-      <c r="F4" s="35" t="s">
-        <v>232</v>
-      </c>
-      <c r="G4" s="35" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="38"/>
       <c r="B5" s="39" t="s">
+        <v>231</v>
+      </c>
+      <c r="C5" s="40" t="s">
+        <v>232</v>
+      </c>
+      <c r="D5" s="39" t="s">
+        <v>233</v>
+      </c>
+      <c r="E5" s="39" t="s">
         <v>234</v>
       </c>
-      <c r="C5" s="40" t="s">
+      <c r="F5" s="41" t="s">
         <v>235</v>
       </c>
-      <c r="D5" s="39" t="s">
+      <c r="G5" s="42" t="s">
         <v>236</v>
-      </c>
-      <c r="E5" s="39" t="s">
-        <v>237</v>
-      </c>
-      <c r="F5" s="41" t="s">
-        <v>238</v>
-      </c>
-      <c r="G5" s="42" t="s">
-        <v>239</v>
       </c>
       <c r="H5" s="38"/>
     </row>
     <row r="6" spans="1:8" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="27"/>
       <c r="B6" s="43" t="s">
+        <v>237</v>
+      </c>
+      <c r="C6" s="44" t="s">
+        <v>238</v>
+      </c>
+      <c r="D6" s="43" t="s">
+        <v>239</v>
+      </c>
+      <c r="E6" s="43" t="s">
         <v>240</v>
       </c>
-      <c r="C6" s="44" t="s">
+      <c r="F6" s="30" t="s">
         <v>241</v>
       </c>
-      <c r="D6" s="43" t="s">
+      <c r="G6" s="45" t="s">
         <v>242</v>
-      </c>
-      <c r="E6" s="43" t="s">
-        <v>243</v>
-      </c>
-      <c r="F6" s="30" t="s">
-        <v>244</v>
-      </c>
-      <c r="G6" s="45" t="s">
-        <v>245</v>
       </c>
       <c r="H6" s="27"/>
     </row>
     <row r="7" spans="1:8" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="46"/>
       <c r="B7" s="47" t="s">
+        <v>243</v>
+      </c>
+      <c r="C7" s="48" t="s">
+        <v>172</v>
+      </c>
+      <c r="D7" s="49" t="s">
+        <v>239</v>
+      </c>
+      <c r="E7" s="49" t="s">
+        <v>244</v>
+      </c>
+      <c r="F7" s="50" t="s">
+        <v>245</v>
+      </c>
+      <c r="G7" s="51" t="s">
         <v>246</v>
-      </c>
-      <c r="C7" s="48" t="s">
-        <v>175</v>
-      </c>
-      <c r="D7" s="49" t="s">
-        <v>242</v>
-      </c>
-      <c r="E7" s="49" t="s">
-        <v>247</v>
-      </c>
-      <c r="F7" s="50" t="s">
-        <v>248</v>
-      </c>
-      <c r="G7" s="51" t="s">
-        <v>249</v>
       </c>
       <c r="H7" s="46"/>
     </row>
     <row r="8" spans="1:8" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="27"/>
       <c r="B8" s="43" t="s">
+        <v>247</v>
+      </c>
+      <c r="C8" s="52" t="s">
+        <v>248</v>
+      </c>
+      <c r="D8" s="43" t="s">
+        <v>239</v>
+      </c>
+      <c r="E8" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="F8" s="30" t="s">
+        <v>249</v>
+      </c>
+      <c r="G8" s="45" t="s">
         <v>250</v>
-      </c>
-      <c r="C8" s="52" t="s">
-        <v>251</v>
-      </c>
-      <c r="D8" s="43" t="s">
-        <v>242</v>
-      </c>
-      <c r="E8" s="43" t="s">
-        <v>243</v>
-      </c>
-      <c r="F8" s="30" t="s">
-        <v>252</v>
-      </c>
-      <c r="G8" s="45" t="s">
-        <v>253</v>
       </c>
       <c r="H8" s="27"/>
     </row>
     <row r="9" spans="1:8" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="53"/>
       <c r="B9" s="54" t="s">
+        <v>251</v>
+      </c>
+      <c r="C9" s="55" t="s">
+        <v>252</v>
+      </c>
+      <c r="D9" s="54" t="s">
+        <v>253</v>
+      </c>
+      <c r="E9" s="54" t="s">
+        <v>244</v>
+      </c>
+      <c r="F9" s="56" t="s">
         <v>254</v>
       </c>
-      <c r="C9" s="55" t="s">
+      <c r="G9" s="57" t="s">
         <v>255</v>
-      </c>
-      <c r="D9" s="54" t="s">
-        <v>256</v>
-      </c>
-      <c r="E9" s="54" t="s">
-        <v>247</v>
-      </c>
-      <c r="F9" s="56" t="s">
-        <v>257</v>
-      </c>
-      <c r="G9" s="57" t="s">
-        <v>258</v>
       </c>
       <c r="H9" s="53"/>
     </row>
     <row r="10" spans="1:8" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="53"/>
       <c r="B10" s="54" t="s">
+        <v>256</v>
+      </c>
+      <c r="C10" s="55" t="s">
+        <v>257</v>
+      </c>
+      <c r="D10" s="54" t="s">
+        <v>258</v>
+      </c>
+      <c r="E10" s="54" t="s">
+        <v>244</v>
+      </c>
+      <c r="F10" s="56" t="s">
         <v>259</v>
       </c>
-      <c r="C10" s="55" t="s">
+      <c r="G10" s="57" t="s">
         <v>260</v>
-      </c>
-      <c r="D10" s="54" t="s">
-        <v>261</v>
-      </c>
-      <c r="E10" s="54" t="s">
-        <v>247</v>
-      </c>
-      <c r="F10" s="56" t="s">
-        <v>262</v>
-      </c>
-      <c r="G10" s="57" t="s">
-        <v>263</v>
       </c>
       <c r="H10" s="53"/>
     </row>
     <row r="11" spans="1:8" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="58"/>
       <c r="B11" s="59" t="s">
+        <v>261</v>
+      </c>
+      <c r="C11" s="60" t="s">
+        <v>262</v>
+      </c>
+      <c r="D11" s="59" t="s">
+        <v>263</v>
+      </c>
+      <c r="E11" s="59" t="s">
+        <v>244</v>
+      </c>
+      <c r="F11" s="61" t="s">
         <v>264</v>
       </c>
-      <c r="C11" s="60" t="s">
+      <c r="G11" s="62" t="s">
         <v>265</v>
-      </c>
-      <c r="D11" s="59" t="s">
-        <v>266</v>
-      </c>
-      <c r="E11" s="59" t="s">
-        <v>247</v>
-      </c>
-      <c r="F11" s="61" t="s">
-        <v>267</v>
-      </c>
-      <c r="G11" s="62" t="s">
-        <v>268</v>
       </c>
       <c r="H11" s="58"/>
     </row>
     <row r="12" spans="1:8" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="58"/>
       <c r="B12" s="59" t="s">
+        <v>266</v>
+      </c>
+      <c r="C12" s="60" t="s">
+        <v>267</v>
+      </c>
+      <c r="D12" s="59" t="s">
+        <v>263</v>
+      </c>
+      <c r="E12" s="59" t="s">
+        <v>244</v>
+      </c>
+      <c r="F12" s="61" t="s">
+        <v>268</v>
+      </c>
+      <c r="G12" s="62" t="s">
         <v>269</v>
-      </c>
-      <c r="C12" s="60" t="s">
-        <v>270</v>
-      </c>
-      <c r="D12" s="59" t="s">
-        <v>266</v>
-      </c>
-      <c r="E12" s="59" t="s">
-        <v>247</v>
-      </c>
-      <c r="F12" s="61" t="s">
-        <v>271</v>
-      </c>
-      <c r="G12" s="62" t="s">
-        <v>272</v>
       </c>
       <c r="H12" s="58"/>
     </row>
     <row r="13" spans="1:8" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="58"/>
       <c r="B13" s="59" t="s">
+        <v>270</v>
+      </c>
+      <c r="C13" s="60" t="s">
+        <v>271</v>
+      </c>
+      <c r="D13" s="59" t="s">
+        <v>263</v>
+      </c>
+      <c r="E13" s="59" t="s">
+        <v>244</v>
+      </c>
+      <c r="F13" s="61" t="s">
+        <v>272</v>
+      </c>
+      <c r="G13" s="62" t="s">
         <v>273</v>
-      </c>
-      <c r="C13" s="60" t="s">
-        <v>274</v>
-      </c>
-      <c r="D13" s="59" t="s">
-        <v>266</v>
-      </c>
-      <c r="E13" s="59" t="s">
-        <v>247</v>
-      </c>
-      <c r="F13" s="61" t="s">
-        <v>275</v>
-      </c>
-      <c r="G13" s="62" t="s">
-        <v>276</v>
       </c>
       <c r="H13" s="58"/>
     </row>
     <row r="14" spans="1:8" ht="31.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="63"/>
       <c r="B14" s="64" t="s">
+        <v>274</v>
+      </c>
+      <c r="C14" s="65" t="s">
+        <v>275</v>
+      </c>
+      <c r="D14" s="64" t="s">
+        <v>258</v>
+      </c>
+      <c r="E14" s="64" t="s">
+        <v>276</v>
+      </c>
+      <c r="F14" s="66" t="s">
         <v>277</v>
       </c>
-      <c r="C14" s="65" t="s">
+      <c r="G14" s="67" t="s">
         <v>278</v>
-      </c>
-      <c r="D14" s="64" t="s">
-        <v>261</v>
-      </c>
-      <c r="E14" s="64" t="s">
-        <v>279</v>
-      </c>
-      <c r="F14" s="66" t="s">
-        <v>280</v>
-      </c>
-      <c r="G14" s="67" t="s">
-        <v>281</v>
       </c>
       <c r="H14" s="63"/>
     </row>
     <row r="16" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="4" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
@@ -3407,96 +3417,96 @@
     </row>
     <row r="17" spans="2:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="3" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
       <c r="E17" s="2" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
     </row>
     <row r="18" spans="2:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="1" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
       <c r="E18" s="72" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="F18" s="72"/>
       <c r="G18" s="72"/>
     </row>
     <row r="19" spans="2:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="73" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C19" s="73"/>
       <c r="D19" s="73"/>
       <c r="E19" s="74" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="F19" s="74"/>
       <c r="G19" s="74"/>
     </row>
     <row r="20" spans="2:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="75" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="C20" s="75"/>
       <c r="D20" s="75"/>
       <c r="E20" s="76" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="F20" s="76"/>
       <c r="G20" s="76"/>
     </row>
     <row r="21" spans="2:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="75" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="C21" s="75"/>
       <c r="D21" s="75"/>
       <c r="E21" s="76" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F21" s="76"/>
       <c r="G21" s="76"/>
     </row>
     <row r="22" spans="2:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="3" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
       <c r="E22" s="2" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
     </row>
     <row r="23" spans="2:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="73" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C23" s="73"/>
       <c r="D23" s="73"/>
       <c r="E23" s="74" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="F23" s="74"/>
       <c r="G23" s="74"/>
     </row>
     <row r="24" spans="2:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="77" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="C24" s="77"/>
       <c r="D24" s="77"/>
       <c r="E24" s="78" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="F24" s="78"/>
       <c r="G24" s="78"/>
@@ -3542,7 +3552,7 @@
   <sheetData>
     <row r="1" spans="2:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B1" s="14" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="C1" s="14"/>
       <c r="D1" s="14"/>
@@ -3550,7 +3560,7 @@
     </row>
     <row r="2" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="13" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>
@@ -3559,7 +3569,7 @@
     <row r="3" spans="2:5" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="2:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="79" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="C4" s="79"/>
       <c r="D4" s="79"/>
@@ -3567,62 +3577,62 @@
     </row>
     <row r="5" spans="2:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="21" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="C5" s="68">
         <v>16</v>
       </c>
       <c r="D5" s="69" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
     </row>
     <row r="6" spans="2:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="21" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="C6" s="68">
         <v>16</v>
       </c>
       <c r="D6" s="69" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
     </row>
     <row r="7" spans="2:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="21" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="C7" s="68">
         <v>32</v>
       </c>
       <c r="D7" s="69" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
     </row>
     <row r="8" spans="2:5" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B8" s="21" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="C8" s="68">
         <v>32767</v>
       </c>
       <c r="D8" s="69" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
     </row>
     <row r="9" spans="2:5" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="21" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="C9" s="68">
         <v>7958</v>
       </c>
       <c r="D9" s="69" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="11" spans="2:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="80" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="C11" s="80"/>
       <c r="D11" s="80"/>
@@ -3630,96 +3640,96 @@
     </row>
     <row r="12" spans="2:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="21" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C12" s="70">
         <f>C8*C9</f>
         <v>260759786</v>
       </c>
       <c r="D12" s="69" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
     </row>
     <row r="13" spans="2:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="29" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="C13" s="70">
         <f>INT(LOG(C8*C9)/LOG(2))+2</f>
         <v>29</v>
       </c>
       <c r="D13" s="71" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
     </row>
     <row r="14" spans="2:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="21" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C14" s="70">
         <f>C7*C8*C9</f>
         <v>8344313152</v>
       </c>
       <c r="D14" s="69" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
     </row>
     <row r="15" spans="2:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="29" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="C15" s="70">
-        <f>INT(LOG(C7*C6*C8)/LOG(2))+2</f>
-        <v>25</v>
+        <f>INT(LOG(C7*C8*C9)/LOG(2))+2</f>
+        <v>34</v>
       </c>
       <c r="D15" s="71" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
     </row>
     <row r="16" spans="2:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="21" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="C16" s="70">
-        <f>INT(LOG(C7*C6*C8)/LOG(2))+9</f>
-        <v>32</v>
+        <f>INT(LOG(C7*C8*C9)/LOG(2))+9</f>
+        <v>41</v>
       </c>
       <c r="D16" s="69" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="29" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="C17" s="70" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="D17" s="71" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="21" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="C18" s="70" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="D18" s="69" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
     </row>
     <row r="19" spans="2:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="29" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="C19" s="70">
         <f>6.02*C5+1.76</f>
         <v>98.08</v>
       </c>
       <c r="D19" s="71" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
   </sheetData>

</xml_diff>